<commit_message>
Elaboração das Tabelas em análise
</commit_message>
<xml_diff>
--- a/Excel/excel-dashboard-financeiro/Dashboard Financeiro/excel-dashboard-financeiro.xlsx
+++ b/Excel/excel-dashboard-financeiro/Dashboard Financeiro/excel-dashboard-financeiro.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12990" windowHeight="5865"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12990" windowHeight="5865" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="CONTAS A PAGAR" sheetId="5" r:id="rId1"/>
@@ -17,7 +17,6 @@
     <sheet name="ANALISES" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="63">
   <si>
     <t>CONTAS A RECEBER</t>
   </si>
@@ -63,13 +62,169 @@
   </si>
   <si>
     <t>CLIENTE</t>
+  </si>
+  <si>
+    <t>Gráfica Rápida</t>
+  </si>
+  <si>
+    <t>Conta de Luz</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>Cartão de Crédito</t>
+  </si>
+  <si>
+    <t>RH</t>
+  </si>
+  <si>
+    <t>Aluguel Imóveis</t>
+  </si>
+  <si>
+    <t>Hospedagem de Site</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Consultoria XPTO</t>
+  </si>
+  <si>
+    <t>Material de Escritório</t>
+  </si>
+  <si>
+    <t>Boleto</t>
+  </si>
+  <si>
+    <t>Vendas</t>
+  </si>
+  <si>
+    <t>Limpeza &amp; Cia</t>
+  </si>
+  <si>
+    <t>Assinatura de Software</t>
+  </si>
+  <si>
+    <t>Energia S.A.</t>
+  </si>
+  <si>
+    <t>Seguro Predial</t>
+  </si>
+  <si>
+    <t>Operacional</t>
+  </si>
+  <si>
+    <t>AWS Amazon</t>
+  </si>
+  <si>
+    <t>Manutenção de Ar-condicionado</t>
+  </si>
+  <si>
+    <t>Campanha de Marketing</t>
+  </si>
+  <si>
+    <t>Administrativo</t>
+  </si>
+  <si>
+    <t>Pix</t>
+  </si>
+  <si>
+    <t>Papelaria Silva</t>
+  </si>
+  <si>
+    <t>Serviços de Consultoria</t>
+  </si>
+  <si>
+    <t>Transferência Bancária</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>Insumos de Produção</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
+  </si>
+  <si>
+    <t>Seguros Porto</t>
+  </si>
+  <si>
+    <t>Limpeza Mensal</t>
+  </si>
+  <si>
+    <t>Internet Fibra</t>
+  </si>
+  <si>
+    <t>Varejo Global</t>
+  </si>
+  <si>
+    <t>Suporte Premium</t>
+  </si>
+  <si>
+    <t>Construtora Alfa</t>
+  </si>
+  <si>
+    <t>Projeto de Software</t>
+  </si>
+  <si>
+    <t>Supermercado Real</t>
+  </si>
+  <si>
+    <t>Venda de Equipamento</t>
+  </si>
+  <si>
+    <t>João Silva</t>
+  </si>
+  <si>
+    <t>Manutenção de Sistema</t>
+  </si>
+  <si>
+    <t>Academia Fit</t>
+  </si>
+  <si>
+    <t>Venda de Licença</t>
+  </si>
+  <si>
+    <t>Escola Aprender</t>
+  </si>
+  <si>
+    <t>Desenvolvimento de Site</t>
+  </si>
+  <si>
+    <t>Hospital Vida</t>
+  </si>
+  <si>
+    <t>Consultoria Técnica</t>
+  </si>
+  <si>
+    <t>Restaurante Sabor</t>
+  </si>
+  <si>
+    <t>Tech Solutions Ltda</t>
+  </si>
+  <si>
+    <t>Prestação de Serviço Mensal</t>
+  </si>
+  <si>
+    <t>Maria Oliveira</t>
+  </si>
+  <si>
+    <t>Curso de Treinamento</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +241,21 @@
     </font>
     <font>
       <sz val="36"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,7 +282,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -120,33 +290,446 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="9"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color theme="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
+  <dxfs count="38">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -154,89 +737,16 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -269,36 +779,24 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -311,6 +809,41 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF9C6500"/>
       </font>
@@ -322,13 +855,45 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -347,27 +912,27 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>262371</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>807893</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>64943</xdr:rowOff>
+      <xdr:rowOff>45893</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1817544</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>232930</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>569768</xdr:rowOff>
+      <xdr:rowOff>550718</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Retângulo Arredondado 1">
+        <xdr:cNvPr id="4" name="Retângulo Arredondado 3">
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3570144" y="64943"/>
+          <a:off x="7672821" y="45893"/>
           <a:ext cx="1565564" cy="504825"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -376,7 +941,9 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg1"/>
+          <a:schemeClr val="accent5">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
         </a:solidFill>
         <a:ln>
           <a:solidFill>
@@ -414,14 +981,8 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>CONTAS A PAGAR</a:t>
+            <a:rPr lang="pt-BR" sz="1600"/>
+            <a:t>ANÁLISES</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -431,27 +992,27 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>395722</xdr:colOff>
+      <xdr:colOff>443968</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>49357</xdr:rowOff>
+      <xdr:rowOff>51148</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>288349</xdr:colOff>
+      <xdr:colOff>336595</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>554182</xdr:rowOff>
+      <xdr:rowOff>555973</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Retângulo Arredondado 2">
+        <xdr:cNvPr id="15" name="Retângulo Arredondado 14">
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5587713" y="49357"/>
-          <a:ext cx="1562100" cy="504825"/>
+          <a:off x="5607175" y="51148"/>
+          <a:ext cx="1548006" cy="504825"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -509,28 +1070,28 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>807893</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>301785</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>45893</xdr:rowOff>
+      <xdr:rowOff>38667</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>232930</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1856958</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>550718</xdr:rowOff>
+      <xdr:rowOff>543492</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Retângulo Arredondado 3">
+        <xdr:cNvPr id="16" name="Retângulo Arredondado 15">
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7672821" y="45893"/>
-          <a:ext cx="1565564" cy="504825"/>
+          <a:off x="3586268" y="38667"/>
+          <a:ext cx="1555173" cy="504825"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -538,9 +1099,7 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="accent5">
-            <a:lumMod val="50000"/>
-          </a:schemeClr>
+          <a:schemeClr val="bg1"/>
         </a:solidFill>
         <a:ln>
           <a:solidFill>
@@ -578,8 +1137,14 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1600"/>
-            <a:t>ANÁLISES</a:t>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>CONTAS A PAGAR</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1090,48 +1655,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="B4:I5" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="B4:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="B4:I31" headerRowDxfId="37" dataDxfId="36">
+  <autoFilter ref="B4:I31"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="DATA DE VENCIMENTO" dataDxfId="20">
+    <tableColumn id="1" name="DATA DE VENCIMENTO" totalsRowLabel="Total" dataDxfId="35" totalsRowDxfId="17">
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" name="FORNECEDOR" dataDxfId="19"/>
-    <tableColumn id="3" name="DESCRIÇÃO" dataDxfId="18"/>
-    <tableColumn id="4" name="VALOR A PAGAR" dataDxfId="17"/>
-    <tableColumn id="5" name="STATUS" dataDxfId="16">
+    <tableColumn id="2" name="FORNECEDOR" dataDxfId="34" totalsRowDxfId="18"/>
+    <tableColumn id="3" name="DESCRIÇÃO" dataDxfId="30" totalsRowDxfId="19"/>
+    <tableColumn id="4" name="VALOR A PAGAR" dataDxfId="28" totalsRowDxfId="20" dataCellStyle="Moeda"/>
+    <tableColumn id="5" name="STATUS" dataDxfId="29" totalsRowDxfId="21">
       <calculatedColumnFormula>IF(G5&lt;&gt;"","PAGO",IF(B5&lt;TODAY(),"ATRASADO","PENDENTE"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" name="DATA DE PAGAMENTO" dataDxfId="15">
+    <tableColumn id="6" name="DATA DE PAGAMENTO" dataDxfId="33" totalsRowDxfId="22">
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="TIPO DE PAGAMENTO" dataDxfId="14"/>
-    <tableColumn id="8" name="CENTRO DE CUSTO" dataDxfId="13"/>
+    <tableColumn id="7" name="TIPO DE PAGAMENTO" dataDxfId="32" totalsRowDxfId="23"/>
+    <tableColumn id="8" name="CENTRO DE CUSTO" totalsRowFunction="count" dataDxfId="31" totalsRowDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela13" displayName="Tabela13" ref="B3:I4" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B3:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tabela4" displayName="Tabela4" ref="B3:I28" totalsRowShown="0" headerRowDxfId="10" dataDxfId="0" tableBorderDxfId="9">
+  <autoFilter ref="B3:I28"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="DATA DE VENCIMENTO" dataDxfId="7">
+    <tableColumn id="1" name="DATA DE VENCIMENTO" dataDxfId="8"/>
+    <tableColumn id="2" name="CLIENTE" dataDxfId="7"/>
+    <tableColumn id="3" name="DESCRIÇÃO" dataDxfId="6"/>
+    <tableColumn id="4" name="VALOR A PAGAR" dataDxfId="5"/>
+    <tableColumn id="5" name="STATUS" dataDxfId="4"/>
+    <tableColumn id="6" name="DATA DE PAGAMENTO" dataDxfId="3">
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" name="CLIENTE" dataDxfId="6"/>
-    <tableColumn id="3" name="DESCRIÇÃO" dataDxfId="5"/>
-    <tableColumn id="4" name="VALOR A PAGAR" dataDxfId="4"/>
-    <tableColumn id="5" name="STATUS" dataDxfId="3">
-      <calculatedColumnFormula>IF(G4&lt;&gt;"","PAGO",IF(B4&lt;TODAY(),"ATRASADO","PENDENTE"))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="6" name="DATA DE PAGAMENTO" dataDxfId="2">
-      <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="TIPO DE PAGAMENTO" dataDxfId="1"/>
-    <tableColumn id="8" name="CENTRO DE CUSTO" dataDxfId="0"/>
+    <tableColumn id="7" name="TIPO DE PAGAMENTO" dataDxfId="2"/>
+    <tableColumn id="8" name="CENTRO DE CUSTO" dataDxfId="1"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1398,13 +1959,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.85546875" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="39.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.42578125" customWidth="1"/>
@@ -1415,73 +1976,731 @@
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="E1" s="7"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <f ca="1">TODAY()</f>
         <v>46222</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4" t="str">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="F5" s="3" t="str">
         <f ca="1">IF(G5&lt;&gt;"","PAGO",IF(B5&lt;TODAY(),"ATRASADO","PENDENTE"))</f>
         <v>PAGO</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <f ca="1">TODAY()</f>
         <v>46222</v>
       </c>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="4">
+        <v>46220</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="6">
+        <v>217311</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="4">
+        <v>46216</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B7" s="4">
+        <v>46208</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="6">
+        <v>452135</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="4">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="4">
+        <v>46217</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="6">
+        <v>155331</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="4">
+        <v>46218</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="4">
+        <v>46171</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="6">
+        <v>65169</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" ref="G9:G11" ca="1" si="0">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="4">
+        <v>46234</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="6">
+        <v>190566</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>46222</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="4">
+        <v>46182</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="6">
+        <v>269948</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>46222</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="4">
+        <v>46240</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="6">
+        <v>498749</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4">
+        <v>46235</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="4">
+        <v>46261</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="6">
+        <v>316793</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4">
+        <v>46261</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="4">
+        <v>46173</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="6">
+        <v>249298</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="4">
+        <v>46174</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="4">
+        <v>46212</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="6">
+        <v>331687</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="4">
+        <v>46208</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="4">
+        <v>46192</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="6">
+        <v>128638</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="4">
+        <f t="shared" ref="G16:G17" ca="1" si="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="4">
+        <v>46220</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="6">
+        <v>256332</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" ca="1" si="1"/>
+        <v>46222</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="4">
+        <v>46211</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="6">
+        <v>407113</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="4">
+        <v>46206</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="4">
+        <v>46202</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="6">
+        <v>474394</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="4">
+        <v>46199</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="4">
+        <v>46232</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="6">
+        <v>35608</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="4">
+        <v>46232</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="4">
+        <v>46178</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="6">
+        <v>457593</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="4">
+        <v>46173</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="4">
+        <v>46264</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="6">
+        <v>306694</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="4">
+        <f t="shared" ref="G22:G24" ca="1" si="2">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="4">
+        <v>46211</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="6">
+        <v>479918</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="4">
+        <f t="shared" ca="1" si="2"/>
+        <v>46222</v>
+      </c>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="4">
+        <v>46248</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="6">
+        <v>357209</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="4">
+        <f t="shared" ca="1" si="2"/>
+        <v>46222</v>
+      </c>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="4">
+        <v>46260</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" s="6">
+        <v>227667</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" s="4">
+        <v>46258</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="4">
+        <v>46252</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" s="6">
+        <v>276131</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="4">
+        <v>46254</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="4">
+        <v>46248</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="6">
+        <v>486368</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="4">
+        <v>46244</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="4">
+        <v>46199</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="6">
+        <v>497059</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="4">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="4">
+        <v>46251</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" s="6">
+        <v>472564</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="4">
+        <v>46250</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="4">
+        <v>46183</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="6">
+        <v>290965</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="4">
+        <f t="shared" ref="G30:G31" ca="1" si="3">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="4">
+        <v>46220</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" s="6">
+        <v>393238</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="4">
+        <f t="shared" ca="1" si="3"/>
+        <v>46222</v>
+      </c>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F5">
-    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
+  <conditionalFormatting sqref="F5:F31">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+      <formula>"PAGO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
+      <formula>"PENDENTE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="3" operator="equal">
       <formula>"ATRASADO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
-      <formula>"PENDENTE"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
-      <formula>"PAGO"</formula>
-    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H31">
       <formula1>"BOLETO,TRANSFERENCIA,PIX,DEBITO,CREDITO,DINHEIRO"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4">
-      <formula1>"MORADIA,ALIMENTAÇÃO,TRANSPORTE,PESSOAL,ADMINISTRATIVO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -1495,7 +2714,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
@@ -1513,68 +2732,680 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="6" t="s">
+    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="7">
+      <c r="B4" s="11">
         <f ca="1">TODAY()</f>
         <v>46222</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6" t="str">
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12" t="str">
         <f ca="1">IF(G4&lt;&gt;"","PAGO",IF(B4&lt;TODAY(),"ATRASADO","PENDENTE"))</f>
         <v>PAGO</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="13">
         <f ca="1">TODAY()</f>
         <v>46222</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="14">
+        <v>46281</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="15">
+        <v>99157</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="16">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="14">
+        <v>46257</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="15">
+        <v>1137025</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="16">
+        <v>46255</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="14">
+        <v>46169</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="15">
+        <v>1001343</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="16">
+        <v>46167</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="14">
+        <v>46273</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="15">
+        <v>374734</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="16">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="14">
+        <v>46261</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="15">
+        <v>971237</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="16">
+        <v>46257</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="14">
+        <v>46167</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="15">
+        <v>1282241</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="16">
+        <v>46169</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="14">
+        <v>46228</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="15">
+        <v>278593</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="16">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="14">
+        <v>46278</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="15">
+        <v>1293239</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="16">
+        <v>46279</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="14">
+        <v>46280</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="15">
+        <v>12266</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="16">
+        <v>46281</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="14">
+        <v>46267</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="15">
+        <v>147901</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="16">
+        <v>46263</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="14">
+        <v>46177</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="15">
+        <v>561159</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="16">
+        <v>46177</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="14">
+        <v>46247</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="15">
+        <v>71884</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="16">
+        <v>46249</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="14">
+        <v>46223</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="15">
+        <v>44260</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="16">
+        <v>46221</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="14">
+        <v>46219</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="15">
+        <v>607481</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="16">
+        <v>46220</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="14">
+        <v>46254</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="15">
+        <v>1337831</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="16">
+        <f ca="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="14">
+        <v>46179</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="15">
+        <v>522722</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="16">
+        <v>46181</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="14">
+        <v>46208</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" s="15">
+        <v>922892</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="16">
+        <v>46207</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="14">
+        <v>46170</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="15">
+        <v>1393655</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="16">
+        <v>46172</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="14">
+        <v>46275</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="15">
+        <v>377976</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="16">
+        <f t="shared" ref="G23:G24" ca="1" si="0">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="14">
+        <v>46263</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="15">
+        <v>1468989</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="16">
+        <f t="shared" ca="1" si="0"/>
+        <v>46222</v>
+      </c>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="14">
+        <v>46232</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="15">
+        <v>643132</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" s="16">
+        <v>46231</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="14">
+        <v>46248</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E26" s="15">
+        <v>890403</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="16">
+        <f t="shared" ref="G26:G28" ca="1" si="1">TODAY()</f>
+        <v>46222</v>
+      </c>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="14">
+        <v>46185</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" s="15">
+        <v>159442</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="16">
+        <f t="shared" ca="1" si="1"/>
+        <v>46222</v>
+      </c>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="14">
+        <v>46176</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" s="15">
+        <v>955553</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="16">
+        <f t="shared" ca="1" si="1"/>
+        <v>46222</v>
+      </c>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F4">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+  <conditionalFormatting sqref="F4:F28">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
       <formula>"PAGO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
       <formula>"PENDENTE"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
       <formula>"ATRASADO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3">
-      <formula1>"MORADIA,ALIMENTAÇÃO,TRANSPORTE,PESSOAL,ADMINISTRATIVO"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H28">
       <formula1>"BOLETO,TRANSFERENCIA,PIX,DEBITO,CREDITO,DINHEIRO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>